<commit_message>
chore: update C04 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -1520,12 +1520,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>公開済</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>差別化ポイント</t>
+          <t>c04-josler-sougou-kousatsu-kakikata.mdx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add C09 article - J-OSLER 29症例の選び方
- New article: c09-josler-byoreki-youyaku-29cases.mdx
- 2 SVG illustrations (balance strategy, 5 conditions)
- OGP slugToMeta entry added
- Backlinks added to b01, b02, c04
- Keyword list status updated
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -1768,10 +1768,14 @@
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>c09-josler-byoreki-youyaku-29cases.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="25" customHeight="1">
       <c r="A27" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update keyword list C06 status to published
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -1640,10 +1640,14 @@
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>c06-josler-nyuingo-keika-kakikata.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="A24" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update A03 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -680,10 +680,14 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>a03-josler-tsukaikata.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="25" customHeight="1">
       <c r="A5" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update G02 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -3308,10 +3308,14 @@
       </c>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J57" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J57" s="2" t="inlineStr">
+        <is>
+          <t>g02-naika-senmoni-itsu-kara.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="25" customHeight="1">
       <c r="A58" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update G03 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -3360,10 +3360,14 @@
       </c>
       <c r="I58" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J58" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>g03-naika-senmoni-sankousho.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="25" customHeight="1">
       <c r="A59" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update J01 status to published in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -4664,12 +4664,12 @@
       </c>
       <c r="I85" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>公開済</t>
         </is>
       </c>
       <c r="J85" s="2" t="inlineStr">
         <is>
-          <t>差別化・内科ナビ連携</t>
+          <t>j01-josler-ai-katsuyo.mdx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
update: J04 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -4824,10 +4824,14 @@
       </c>
       <c r="I88" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J88" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>j04-josler-jitan.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="89" ht="25" customHeight="1">
       <c r="A89" s="2" t="inlineStr">

</xml_diff>

<commit_message>
update: D02 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -2048,10 +2048,14 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>d02-josler-byoreki-youyaku-junkanki.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="25" customHeight="1">
       <c r="A32" s="2" t="inlineStr">

</xml_diff>

<commit_message>
update: D03 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -2100,10 +2100,14 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>d03-josler-byoreki-youyaku-kokyuuki.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="25" customHeight="1">
       <c r="A33" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update B06 status to 公開済 in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -1244,10 +1244,14 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>b06-josler-jiko-shousatsu-kakikata.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="25" customHeight="1">
       <c r="A16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: update N08 and E01 status in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -2760,12 +2760,12 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
           <t>e01-josler-shinchoku-kanri.mdx</t>
-        </is>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>ツール連携</t>
         </is>
       </c>
     </row>
@@ -8163,12 +8163,12 @@
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>公開済</t>
         </is>
       </c>
       <c r="J156" t="inlineStr">
         <is>
-          <t>初期研修医の入口記事</t>
+          <t>n08-senkoui-program-erabikata.mdx</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: update B04 status in keyword list
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -1144,10 +1144,14 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J13" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>b04-josler-shikkanngun-ichiran.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="25" customHeight="1">
       <c r="A14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore: OGP titleMap + キーワードリスト更新（G06,G07,B07,C10,C11）
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -1300,7 +1300,7 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>b07-josler-shourei-touroku-shounin-sarenai.mdx</t>
         </is>
       </c>
       <c r="J16" s="2" t="n"/>
@@ -1860,7 +1860,7 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>c10-josler-accept-reject.mdx</t>
         </is>
       </c>
       <c r="J27" s="2" t="n"/>
@@ -1908,7 +1908,7 @@
       </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>c11-josler-ichijihyouka.mdx</t>
         </is>
       </c>
       <c r="J28" s="2" t="n"/>
@@ -3576,7 +3576,7 @@
       </c>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>g06-naika-senmoni-goukakuritsu.mdx</t>
         </is>
       </c>
       <c r="J61" s="2" t="n"/>
@@ -3624,7 +3624,7 @@
       </c>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
+          <t>g07-naika-senmoni-nanido.mdx</t>
         </is>
       </c>
       <c r="J62" s="2" t="n"/>

</xml_diff>

<commit_message>
Update keyword list: D11, D12, D14 published
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -2528,10 +2528,14 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="n"/>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>d11-josler-byoreki-youyaku-kyuukyuu.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="25" customHeight="1">
       <c r="A41" s="2" t="inlineStr">
@@ -2576,10 +2580,14 @@
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="n"/>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>d12-josler-geka-shoukai-shourei.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="25" customHeight="1">
       <c r="A42" s="2" t="inlineStr">
@@ -2672,10 +2680,14 @@
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J43" s="2" t="n"/>
+          <t>published</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>d14-josler-gairai-shourei.mdx</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="25" customHeight="1">
       <c r="A44" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add F04: J-OSLER e-Learningの受講方法
- 共通講習3分野（医療倫理・安全・感染対策）のe-Learning受講手順
- 内科オンデマンドの登録・受講・修了証取得の流れ
- J-OSLERへの反映方法、費用（2,200円/講座）
- OGPエントリ追加、a06にバックリンク追加
- キーワードリスト更新（F04 → 公開済）

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/keywords/naikanavi_keyword_list.xlsx
+++ b/docs/keywords/naikanavi_keyword_list.xlsx
@@ -3248,10 +3248,14 @@
       </c>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>未着手</t>
-        </is>
-      </c>
-      <c r="J54" s="2" t="n"/>
+          <t>公開済</t>
+        </is>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>f04-josler-e-learning</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="25" customHeight="1">
       <c r="A55" s="2" t="inlineStr">

</xml_diff>